<commit_message>
auto-publish commission xlsx: payments upload (1 months)
</commit_message>
<xml_diff>
--- a/commission/karin/2026-08.xlsx
+++ b/commission/karin/2026-08.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="57">
   <si>
     <t>Equine Performance Labs, LLC</t>
   </si>
@@ -37,6 +37,12 @@
     <t>Q3 Route C Accelerator — tiered on invoiced revenue when $30K gate met (else standard waterfall)</t>
   </si>
   <si>
+    <t>Basis</t>
+  </si>
+  <si>
+    <t>✅ CRM + QuickBooks reconciled (paid on cleared)</t>
+  </si>
+  <si>
     <t>Route C — Q3 Accelerator</t>
   </si>
   <si>
@@ -49,19 +55,19 @@
     <t>New / Reactivated (15%)</t>
   </si>
   <si>
-    <t>on $21,900.00 collected</t>
+    <t>on $17,100.00 collected</t>
   </si>
   <si>
     <t>Growth above baseline (12.5%)</t>
   </si>
   <si>
-    <t>on $13,463.64 collected</t>
+    <t>on $12,363.64 collected</t>
   </si>
   <si>
     <t>Baseline reorders (10%)</t>
   </si>
   <si>
-    <t>on $6,936.36 collected</t>
+    <t>on $8,036.36 collected</t>
   </si>
   <si>
     <t>Spiff — 2 new acct(s) × $750</t>
@@ -73,7 +79,7 @@
     <t>vs. standard waterfall would have paid</t>
   </si>
   <si>
-    <t>Uplift: $6746.59</t>
+    <t>Uplift: $6239.09</t>
   </si>
   <si>
     <t>Account / Date</t>
@@ -142,12 +148,6 @@
     <t>ORD-EPL-1189</t>
   </si>
   <si>
-    <t>Smith Performance Equine</t>
-  </si>
-  <si>
-    <t>ORD-EPL-1183</t>
-  </si>
-  <si>
     <t>Signature Equine Hospital</t>
   </si>
   <si>
@@ -157,13 +157,10 @@
     <t>Elgin Equine</t>
   </si>
   <si>
+    <t>ORD-EPL-1185</t>
+  </si>
+  <si>
     <t>ORD-EPL-1129</t>
-  </si>
-  <si>
-    <t>Panorama Equine Medical and Surgical Center</t>
-  </si>
-  <si>
-    <t>ORD-EPL-1157</t>
   </si>
   <si>
     <t>Buffalo Veterinary Clinic PC</t>
@@ -229,6 +226,11 @@
     <font>
       <b/>
       <color rgb="0F5E4F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="0F5E4F"/>
       <sz val="12"/>
     </font>
     <font>
@@ -257,11 +259,6 @@
     <font>
       <b/>
       <color rgb="FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="0F5E4F"/>
       <sz val="10"/>
     </font>
     <font>
@@ -306,7 +303,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -314,23 +311,24 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -690,7 +688,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
@@ -711,7 +709,7 @@
         <v>1</v>
       </c>
       <c r="H1" s="3">
-        <v>9161.59</v>
+        <v>8414.09</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -736,549 +734,515 @@
         <v>7</v>
       </c>
     </row>
+    <row r="4" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
-        <v>8</v>
+      <c r="A5" s="7" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="7">
+        <v>11</v>
+      </c>
+      <c r="B6" s="8">
         <v>78375</v>
       </c>
-      <c r="C6" s="8" t="s">
-        <v>10</v>
+      <c r="C6" s="9" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="9">
-        <v>3285</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="B7" s="10">
+        <v>2565</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="9">
-        <v>1682.95</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="B8" s="10">
+        <v>1545.45</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="9">
-        <v>693.64</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="B9" s="10">
+        <v>803.64</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" s="9">
+        <v>19</v>
+      </c>
+      <c r="B10" s="10">
         <v>1500</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="9">
+        <v>20</v>
+      </c>
+      <c r="B11" s="10">
         <v>2000</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" s="11">
-        <v>2415</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>20</v>
+      <c r="A12" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="12">
+        <v>2175</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14" s="13" t="s">
+      <c r="A14" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="B14" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="C14" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="F14" s="14" t="s">
+      <c r="D14" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="G14" s="14" t="s">
+      <c r="E14" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="H14" s="14" t="s">
+      <c r="F14" s="15" t="s">
         <v>28</v>
       </c>
+      <c r="G14" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="H14" s="15" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="F15" s="16">
+      <c r="A15" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="F15" s="17">
         <v>10500</v>
       </c>
-      <c r="H15" s="17">
+      <c r="H15" s="18">
         <v>1575</v>
       </c>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B16" s="18">
+      <c r="B16" s="19">
         <v>46262.5</v>
       </c>
-      <c r="C16" s="19" t="s">
-        <v>30</v>
+      <c r="C16" s="20" t="s">
+        <v>32</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F16" s="20">
+        <v>33</v>
+      </c>
+      <c r="F16" s="21">
         <v>10500</v>
       </c>
-      <c r="G16" s="21">
+      <c r="G16" s="22">
         <v>0.15</v>
       </c>
-      <c r="H16" s="22">
+      <c r="H16" s="23">
         <v>1575</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="F18" s="16">
+      <c r="A18" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="F18" s="17">
         <v>7200</v>
       </c>
-      <c r="H18" s="17">
+      <c r="H18" s="18">
         <v>829.09</v>
       </c>
     </row>
     <row r="19" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B19" s="18">
+      <c r="B19" s="19">
         <v>46254.5</v>
       </c>
-      <c r="C19" s="19" t="s">
-        <v>30</v>
+      <c r="C19" s="20" t="s">
+        <v>32</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F19" s="20">
+        <v>35</v>
+      </c>
+      <c r="F19" s="21">
         <v>1800</v>
       </c>
-      <c r="G19" s="21">
+      <c r="G19" s="22">
         <v>0.11515151515151516</v>
       </c>
-      <c r="H19" s="22">
+      <c r="H19" s="23">
         <v>207.27</v>
       </c>
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B20" s="18">
+      <c r="B20" s="19">
         <v>46254.5</v>
       </c>
-      <c r="C20" s="19" t="s">
-        <v>30</v>
+      <c r="C20" s="20" t="s">
+        <v>32</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="F20" s="20">
+        <v>36</v>
+      </c>
+      <c r="F20" s="21">
         <v>2400</v>
       </c>
-      <c r="G20" s="21">
+      <c r="G20" s="22">
         <v>0.11515151515151516</v>
       </c>
-      <c r="H20" s="22">
+      <c r="H20" s="23">
         <v>276.36</v>
       </c>
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B21" s="18">
+      <c r="B21" s="19">
         <v>46261.5</v>
       </c>
-      <c r="C21" s="19" t="s">
-        <v>30</v>
+      <c r="C21" s="20" t="s">
+        <v>32</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F21" s="20">
+        <v>37</v>
+      </c>
+      <c r="F21" s="21">
         <v>600</v>
       </c>
-      <c r="G21" s="21">
+      <c r="G21" s="22">
         <v>0.11515151515151516</v>
       </c>
-      <c r="H21" s="22">
+      <c r="H21" s="23">
         <v>69.09</v>
       </c>
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B22" s="18">
+      <c r="B22" s="19">
         <v>46261.5</v>
       </c>
-      <c r="C22" s="19" t="s">
-        <v>30</v>
+      <c r="C22" s="20" t="s">
+        <v>32</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F22" s="20">
+        <v>38</v>
+      </c>
+      <c r="F22" s="21">
         <v>2400</v>
       </c>
-      <c r="G22" s="21">
+      <c r="G22" s="22">
         <v>0.11515151515151516</v>
       </c>
-      <c r="H22" s="22">
+      <c r="H22" s="23">
         <v>276.36</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="F24" s="16">
+      <c r="A24" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="F24" s="17">
         <v>4800</v>
       </c>
-      <c r="H24" s="17">
+      <c r="H24" s="18">
         <v>480</v>
       </c>
     </row>
     <row r="25" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B25" s="18">
+      <c r="B25" s="19">
         <v>46239.5</v>
       </c>
-      <c r="C25" s="19" t="s">
-        <v>30</v>
+      <c r="C25" s="20" t="s">
+        <v>32</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F25" s="20">
+        <v>40</v>
+      </c>
+      <c r="F25" s="21">
         <v>4800</v>
       </c>
-      <c r="G25" s="21">
+      <c r="G25" s="22">
         <v>0.1</v>
       </c>
-      <c r="H25" s="22">
+      <c r="H25" s="23">
         <v>480</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="F27" s="16">
+      <c r="A27" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="F27" s="17">
         <v>4800</v>
       </c>
-      <c r="H27" s="17">
+      <c r="H27" s="18">
         <v>720</v>
       </c>
     </row>
     <row r="28" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B28" s="18">
+      <c r="B28" s="19">
         <v>46254.5</v>
       </c>
-      <c r="C28" s="19" t="s">
-        <v>30</v>
+      <c r="C28" s="20" t="s">
+        <v>32</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="F28" s="20">
+        <v>42</v>
+      </c>
+      <c r="F28" s="21">
         <v>4800</v>
       </c>
-      <c r="G28" s="21">
+      <c r="G28" s="22">
         <v>0.15</v>
       </c>
-      <c r="H28" s="22">
+      <c r="H28" s="23">
         <v>720</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="F30" s="16">
+      <c r="A30" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="F30" s="17">
         <v>4800</v>
       </c>
-      <c r="H30" s="17">
+      <c r="H30" s="18">
         <v>576</v>
       </c>
     </row>
     <row r="31" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B31" s="18">
+      <c r="B31" s="19">
         <v>46254.5</v>
       </c>
-      <c r="C31" s="19" t="s">
-        <v>30</v>
+      <c r="C31" s="20" t="s">
+        <v>32</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F31" s="20">
+        <v>44</v>
+      </c>
+      <c r="F31" s="21">
         <v>4800</v>
       </c>
-      <c r="G31" s="21">
+      <c r="G31" s="22">
         <v>0.12000000000000001</v>
       </c>
-      <c r="H31" s="22">
+      <c r="H31" s="23">
         <v>576</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="F33" s="16">
+      <c r="A33" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="F33" s="17">
         <v>4800</v>
       </c>
-      <c r="H33" s="17">
-        <v>720</v>
+      <c r="H33" s="18">
+        <v>584</v>
       </c>
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B34" s="18">
+      <c r="B34" s="19">
         <v>46259.5</v>
       </c>
-      <c r="C34" s="19" t="s">
-        <v>30</v>
+      <c r="C34" s="20" t="s">
+        <v>32</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="F34" s="20">
+        <v>46</v>
+      </c>
+      <c r="F34" s="21">
         <v>4800</v>
       </c>
-      <c r="G34" s="21">
+      <c r="G34" s="22">
+        <v>0.12166666666666666</v>
+      </c>
+      <c r="H34" s="23">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="F36" s="17">
+        <v>3600</v>
+      </c>
+      <c r="H36" s="18">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="37" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B37" s="19">
+        <v>46254.5</v>
+      </c>
+      <c r="C37" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F37" s="21">
+        <v>1800</v>
+      </c>
+      <c r="G37" s="22">
+        <v>0.1</v>
+      </c>
+      <c r="H37" s="23">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="38" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B38" s="19">
+        <v>46254.5</v>
+      </c>
+      <c r="C38" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F38" s="21">
+        <v>1800</v>
+      </c>
+      <c r="G38" s="22">
+        <v>0.1</v>
+      </c>
+      <c r="H38" s="23">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="F40" s="17">
+        <v>1200</v>
+      </c>
+      <c r="H40" s="18">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B41" s="19">
+        <v>46244.5</v>
+      </c>
+      <c r="C41" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F41" s="21">
+        <v>1200</v>
+      </c>
+      <c r="G41" s="22">
+        <v>0.1</v>
+      </c>
+      <c r="H41" s="23">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="F43" s="17">
+        <v>1200</v>
+      </c>
+      <c r="H43" s="18">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="44" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B44" s="19">
+        <v>46262.5</v>
+      </c>
+      <c r="C44" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F44" s="21">
+        <v>1200</v>
+      </c>
+      <c r="G44" s="22">
         <v>0.15</v>
       </c>
-      <c r="H34" s="22">
-        <v>720</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="F36" s="16">
-        <v>4800</v>
-      </c>
-      <c r="H36" s="17">
-        <v>584</v>
-      </c>
-    </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B37" s="18">
-        <v>46259.5</v>
-      </c>
-      <c r="C37" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F37" s="20">
-        <v>4800</v>
-      </c>
-      <c r="G37" s="21">
-        <v>0.12166666666666666</v>
-      </c>
-      <c r="H37" s="22">
-        <v>584</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="F39" s="16">
-        <v>1800</v>
-      </c>
-      <c r="H39" s="17">
+      <c r="H44" s="23">
         <v>180</v>
       </c>
     </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B40" s="18">
-        <v>46254.5</v>
-      </c>
-      <c r="C40" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F40" s="20">
-        <v>1800</v>
-      </c>
-      <c r="G40" s="21">
-        <v>0.1</v>
-      </c>
-      <c r="H40" s="22">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="F42" s="16">
-        <v>1800</v>
-      </c>
-      <c r="H42" s="17">
-        <v>207.5</v>
-      </c>
-    </row>
-    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B43" s="18">
-        <v>46259.5</v>
-      </c>
-      <c r="C43" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="F43" s="20">
-        <v>1800</v>
-      </c>
-      <c r="G43" s="21">
-        <v>0.11527777777777777</v>
-      </c>
-      <c r="H43" s="22">
-        <v>207.5</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A45" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="F45" s="16">
-        <v>1200</v>
-      </c>
-      <c r="H45" s="17">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="46" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B46" s="18">
-        <v>46244.5</v>
-      </c>
-      <c r="C46" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="F46" s="20">
-        <v>1200</v>
-      </c>
-      <c r="G46" s="21">
-        <v>0.1</v>
-      </c>
-      <c r="H46" s="22">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A48" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="F48" s="16">
-        <v>1200</v>
-      </c>
-      <c r="H48" s="17">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B49" s="18">
-        <v>46262.5</v>
-      </c>
-      <c r="C49" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="E49" s="2" t="s">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="F49" s="20">
-        <v>1200</v>
-      </c>
-      <c r="G49" s="21">
+      <c r="F46" s="17">
+        <v>600</v>
+      </c>
+      <c r="H46" s="18">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="47" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B47" s="19">
+        <v>46252.5</v>
+      </c>
+      <c r="C47" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F47" s="21">
+        <v>600</v>
+      </c>
+      <c r="G47" s="22">
         <v>0.15</v>
       </c>
-      <c r="H49" s="22">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A51" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="F51" s="16">
-        <v>600</v>
-      </c>
-      <c r="H51" s="17">
+      <c r="H47" s="23">
         <v>90</v>
       </c>
     </row>
-    <row r="52" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B52" s="18">
-        <v>46252.5</v>
-      </c>
-      <c r="C52" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="E52" s="2" t="s">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="F52" s="20">
-        <v>600</v>
-      </c>
-      <c r="G52" s="21">
-        <v>0.15</v>
-      </c>
-      <c r="H52" s="22">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A55" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="F55" s="24">
+      <c r="F50" s="25">
         <v>78375</v>
       </c>
-      <c r="H55" s="25">
-        <v>9161.59</v>
+      <c r="H50" s="26">
+        <v>8414.09</v>
       </c>
     </row>
   </sheetData>

</xml_diff>